<commit_message>
Added LPF/BPF/HPF made folders
</commit_message>
<xml_diff>
--- a/Gain Sheet.xlsx
+++ b/Gain Sheet.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KUSH\ArtixMix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D968A580-A7A7-4540-A3B4-A45EA15C3F47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A4B57C2-0A2E-4D79-97F8-36E94335CF43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{162F6800-650B-40DC-87AA-5313FF53ABEB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{162F6800-650B-40DC-87AA-5313FF53ABEB}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Vol Control" sheetId="1" r:id="rId1"/>
+    <sheet name="Filters" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="51">
   <si>
     <t>Amplitude Ratio</t>
   </si>
@@ -105,19 +106,111 @@
   </si>
   <si>
     <t xml:space="preserve">Error </t>
+  </si>
+  <si>
+    <t>Sr. No</t>
+  </si>
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>Hex</t>
+  </si>
+  <si>
+    <t>Roubnded off</t>
+  </si>
+  <si>
+    <t>Amp Ratio</t>
+  </si>
+  <si>
+    <t>Error</t>
+  </si>
+  <si>
+    <t>Input from ADC</t>
+  </si>
+  <si>
+    <t>Input from SDC</t>
+  </si>
+  <si>
+    <t>Theory</t>
+  </si>
+  <si>
+    <t>16 Bit</t>
+  </si>
+  <si>
+    <t>24 Bit</t>
+  </si>
+  <si>
+    <t>Number * 2^16</t>
+  </si>
+  <si>
+    <t>0F36C</t>
+  </si>
+  <si>
+    <t>Co efficient</t>
+  </si>
+  <si>
+    <t>Zero</t>
+  </si>
+  <si>
+    <t>Pole</t>
+  </si>
+  <si>
+    <t>20CE5</t>
+  </si>
+  <si>
+    <t>0AAA9</t>
+  </si>
+  <si>
+    <t>0729B</t>
+  </si>
+  <si>
+    <t>2C7F8</t>
+  </si>
+  <si>
+    <t>2AAAE</t>
+  </si>
+  <si>
+    <t>LPF</t>
+  </si>
+  <si>
+    <t>HPF</t>
+  </si>
+  <si>
+    <t>4K</t>
+  </si>
+  <si>
+    <t>BPF</t>
+  </si>
+  <si>
+    <t>0F9A2</t>
+  </si>
+  <si>
+    <t>01D49</t>
+  </si>
+  <si>
+    <t>00EA5</t>
+  </si>
+  <si>
+    <t>20CBC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -140,10 +233,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -478,8 +574,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30640A05-FE0D-4691-B386-01EF647E2A68}">
-  <dimension ref="A1:M14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:S17"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="8.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.6640625" bestFit="1" customWidth="1"/>
@@ -490,9 +586,10 @@
     <col min="8" max="9" width="5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6.44140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -526,8 +623,23 @@
       <c r="M1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O1" t="s">
+        <v>28</v>
+      </c>
+      <c r="P1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>20</v>
+      </c>
+      <c r="R1" t="s">
+        <v>26</v>
+      </c>
+      <c r="S1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19">
       <c r="A2">
         <v>-6</v>
       </c>
@@ -564,8 +676,25 @@
         <f>(K2-B2)*100/B2</f>
         <v>-4.4580506783714856E-2</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O2">
+        <v>316</v>
+      </c>
+      <c r="P2">
+        <v>1048576</v>
+      </c>
+      <c r="Q2">
+        <v>525536</v>
+      </c>
+      <c r="R2">
+        <f>Q2/P2</f>
+        <v>0.501190185546875</v>
+      </c>
+      <c r="S2">
+        <f>(R2-B2)*100</f>
+        <v>-9.8144531249788614E-4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19">
       <c r="A3">
         <v>-5</v>
       </c>
@@ -602,8 +731,25 @@
         <f t="shared" ref="M3:M14" si="2">(K3-B3)*100/B3</f>
         <v>-7.8500133380796765E-3</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O3">
+        <v>631</v>
+      </c>
+      <c r="P3">
+        <v>1048576</v>
+      </c>
+      <c r="Q3">
+        <v>589600</v>
+      </c>
+      <c r="R3">
+        <f t="shared" ref="R3:R14" si="3">Q3/P3</f>
+        <v>0.562286376953125</v>
+      </c>
+      <c r="S3">
+        <f t="shared" ref="S3:S14" si="4">(R3-B3)*100</f>
+        <v>-1.3623046875022027E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19">
       <c r="A4">
         <v>-4</v>
       </c>
@@ -640,8 +786,25 @@
         <f t="shared" si="2"/>
         <v>-2.2286053882726677E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O4">
+        <v>946</v>
+      </c>
+      <c r="P4">
+        <v>1048576</v>
+      </c>
+      <c r="Q4">
+        <v>661664</v>
+      </c>
+      <c r="R4">
+        <f t="shared" si="3"/>
+        <v>0.631011962890625</v>
+      </c>
+      <c r="S4">
+        <f t="shared" si="4"/>
+        <v>1.1962890624994671E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19">
       <c r="A5">
         <v>-3</v>
       </c>
@@ -678,8 +841,25 @@
         <f t="shared" si="2"/>
         <v>-1.9258104958323734E-2</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O5">
+        <v>1261</v>
+      </c>
+      <c r="P5">
+        <v>1048576</v>
+      </c>
+      <c r="Q5">
+        <v>742272</v>
+      </c>
+      <c r="R5">
+        <f t="shared" si="3"/>
+        <v>0.7078857421875</v>
+      </c>
+      <c r="S5">
+        <f t="shared" si="4"/>
+        <v>-1.425781249997371E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19">
       <c r="A6">
         <v>-2</v>
       </c>
@@ -716,8 +896,25 @@
         <f t="shared" si="2"/>
         <v>-1.3917521717236063E-2</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O6">
+        <v>1576</v>
+      </c>
+      <c r="P6">
+        <v>1048576</v>
+      </c>
+      <c r="Q6">
+        <v>832896</v>
+      </c>
+      <c r="R6">
+        <f t="shared" si="3"/>
+        <v>0.7943115234375</v>
+      </c>
+      <c r="S6">
+        <f t="shared" si="4"/>
+        <v>1.152343749999396E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19">
       <c r="A7">
         <v>-1</v>
       </c>
@@ -754,8 +951,25 @@
         <f t="shared" si="2"/>
         <v>-0.45921336811398872</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O7">
+        <v>1891</v>
+      </c>
+      <c r="P7">
+        <v>1048576</v>
+      </c>
+      <c r="Q7">
+        <v>930496</v>
+      </c>
+      <c r="R7">
+        <f t="shared" si="3"/>
+        <v>0.88739013671875</v>
+      </c>
+      <c r="S7">
+        <f t="shared" si="4"/>
+        <v>-0.39098632812499812</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19">
       <c r="A8">
         <v>0</v>
       </c>
@@ -792,8 +1006,25 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O8">
+        <v>2206</v>
+      </c>
+      <c r="P8">
+        <v>1048576</v>
+      </c>
+      <c r="Q8">
+        <v>1048576</v>
+      </c>
+      <c r="R8">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="S8">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19">
       <c r="A9">
         <v>1</v>
       </c>
@@ -807,7 +1038,7 @@
         <v>9</v>
       </c>
       <c r="E9">
-        <f t="shared" ref="E9:E14" si="3">B9*32768</f>
+        <f t="shared" ref="E9:E14" si="5">B9*32768</f>
         <v>36765.696000000004</v>
       </c>
       <c r="F9">
@@ -830,8 +1061,25 @@
         <f t="shared" si="2"/>
         <v>0.15858260918002598</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O9">
+        <v>2521</v>
+      </c>
+      <c r="P9">
+        <v>1048576</v>
+      </c>
+      <c r="Q9">
+        <v>1178560</v>
+      </c>
+      <c r="R9">
+        <f t="shared" si="3"/>
+        <v>1.12396240234375</v>
+      </c>
+      <c r="S9">
+        <f t="shared" si="4"/>
+        <v>0.19624023437498916</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19">
       <c r="A10">
         <v>2</v>
       </c>
@@ -845,7 +1093,7 @@
         <v>10</v>
       </c>
       <c r="E10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>41251.635199999997</v>
       </c>
       <c r="F10">
@@ -868,8 +1116,25 @@
         <f t="shared" si="2"/>
         <v>-8.8122567320603699E-3</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O10">
+        <v>2836</v>
+      </c>
+      <c r="P10">
+        <v>1048576</v>
+      </c>
+      <c r="Q10">
+        <v>1320064</v>
+      </c>
+      <c r="R10">
+        <f t="shared" si="3"/>
+        <v>1.2589111328125</v>
+      </c>
+      <c r="S10">
+        <f t="shared" si="4"/>
+        <v>1.1132812500092015E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19">
       <c r="A11">
         <v>3</v>
       </c>
@@ -883,7 +1148,7 @@
         <v>11</v>
       </c>
       <c r="E11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>46284.800000000003</v>
       </c>
       <c r="F11">
@@ -906,8 +1171,25 @@
         <f t="shared" si="2"/>
         <v>0.1279037610619406</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O11">
+        <v>3150</v>
+      </c>
+      <c r="P11">
+        <v>1048576</v>
+      </c>
+      <c r="Q11">
+        <v>1483168</v>
+      </c>
+      <c r="R11">
+        <f t="shared" si="3"/>
+        <v>1.414459228515625</v>
+      </c>
+      <c r="S11">
+        <f t="shared" si="4"/>
+        <v>0.19592285156249112</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19">
       <c r="A12">
         <v>4</v>
       </c>
@@ -921,7 +1203,7 @@
         <v>12</v>
       </c>
       <c r="E12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>51934.003199999999</v>
       </c>
       <c r="F12">
@@ -944,8 +1226,25 @@
         <f t="shared" si="2"/>
         <v>-1.1559286074829674E-2</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O12">
+        <v>3466</v>
+      </c>
+      <c r="P12">
+        <v>1048576</v>
+      </c>
+      <c r="Q12">
+        <v>1661888</v>
+      </c>
+      <c r="R12">
+        <f t="shared" si="3"/>
+        <v>1.58489990234375</v>
+      </c>
+      <c r="S12">
+        <f t="shared" si="4"/>
+        <v>-9.7656249975486276E-6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19">
       <c r="A13">
         <v>5</v>
       </c>
@@ -959,7 +1258,7 @@
         <v>13</v>
       </c>
       <c r="E13">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>58271.3344</v>
       </c>
       <c r="F13">
@@ -982,8 +1281,25 @@
         <f t="shared" si="2"/>
         <v>-1.258663470730427E-2</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O13">
+        <v>3781</v>
+      </c>
+      <c r="P13">
+        <v>1048576</v>
+      </c>
+      <c r="Q13">
+        <v>1864672</v>
+      </c>
+      <c r="R13">
+        <f t="shared" si="3"/>
+        <v>1.778289794921875</v>
+      </c>
+      <c r="S13">
+        <f t="shared" si="4"/>
+        <v>-1.0205078124991829E-3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19">
       <c r="A14">
         <v>6</v>
       </c>
@@ -997,7 +1313,7 @@
         <v>14</v>
       </c>
       <c r="E14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>65381.990400000002</v>
       </c>
       <c r="F14">
@@ -1020,8 +1336,663 @@
         <f t="shared" si="2"/>
         <v>-9.1621560667605635E-3</v>
       </c>
+      <c r="O14">
+        <v>4095</v>
+      </c>
+      <c r="P14">
+        <v>1048576</v>
+      </c>
+      <c r="Q14">
+        <v>2092224</v>
+      </c>
+      <c r="R14">
+        <f t="shared" si="3"/>
+        <v>1.99530029296875</v>
+      </c>
+      <c r="S14">
+        <f t="shared" si="4"/>
+        <v>2.9296874992645883E-5</v>
+      </c>
+    </row>
+    <row r="17" spans="3:17">
+      <c r="C17" t="s">
+        <v>30</v>
+      </c>
+      <c r="K17" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>32</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{576ACB22-FE3C-4C68-B871-26C12037A2C8}">
+  <dimension ref="A1:M22"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="4.109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="4.109375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K1" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>3.0935400000000002E-4</v>
+      </c>
+      <c r="C2">
+        <f>B2*65536</f>
+        <v>20.273823744000001</v>
+      </c>
+      <c r="D2">
+        <v>20</v>
+      </c>
+      <c r="E2">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>0.66663827521715202</v>
+      </c>
+      <c r="J2">
+        <f t="shared" ref="J2:J7" si="0">I2*2^16</f>
+        <v>43688.806004631275</v>
+      </c>
+      <c r="K2">
+        <v>43689</v>
+      </c>
+      <c r="L2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>6.1870800000000004E-4</v>
+      </c>
+      <c r="C3">
+        <f t="shared" ref="C3:C7" si="1">B3*65536</f>
+        <v>40.547647488000003</v>
+      </c>
+      <c r="D3">
+        <v>40</v>
+      </c>
+      <c r="E3">
+        <v>28</v>
+      </c>
+      <c r="F3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>-1.3332765504343</v>
+      </c>
+      <c r="J3">
+        <f t="shared" si="0"/>
+        <v>-87377.612009262288</v>
+      </c>
+      <c r="K3">
+        <v>-87378</v>
+      </c>
+      <c r="L3" t="s">
+        <v>42</v>
+      </c>
+      <c r="M3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>3.0935400000000002E-4</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="1"/>
+        <v>20.273823744000001</v>
+      </c>
+      <c r="D4">
+        <v>20</v>
+      </c>
+      <c r="E4">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4">
+        <v>3</v>
+      </c>
+      <c r="I4">
+        <v>0.66663827521715202</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="0"/>
+        <v>43688.806004631275</v>
+      </c>
+      <c r="K4">
+        <v>43689</v>
+      </c>
+      <c r="L4" t="s">
+        <v>39</v>
+      </c>
+      <c r="M4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="1"/>
+        <v>65536</v>
+      </c>
+      <c r="D5">
+        <v>65536</v>
+      </c>
+      <c r="E5">
+        <v>10000</v>
+      </c>
+      <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H5">
+        <v>4</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="0"/>
+        <v>65536</v>
+      </c>
+      <c r="K5">
+        <v>65536</v>
+      </c>
+      <c r="L5">
+        <v>10000</v>
+      </c>
+      <c r="M5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>-1.9496374000000001</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="1"/>
+        <v>-127771.4366464</v>
+      </c>
+      <c r="D6">
+        <v>-127771</v>
+      </c>
+      <c r="E6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>-1.2188761083637001</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="0"/>
+        <v>-79880.264637723449</v>
+      </c>
+      <c r="K6">
+        <v>-79880</v>
+      </c>
+      <c r="L6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>0.95087489999999997</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="1"/>
+        <v>62316.537446399998</v>
+      </c>
+      <c r="D7">
+        <v>62316</v>
+      </c>
+      <c r="E7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H7">
+        <v>6</v>
+      </c>
+      <c r="I7">
+        <v>0.447676992504908</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="0"/>
+        <v>29338.959380801651</v>
+      </c>
+      <c r="K7">
+        <v>29339</v>
+      </c>
+      <c r="L7" t="s">
+        <v>40</v>
+      </c>
+      <c r="M7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="D10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10">
+        <v>250</v>
+      </c>
+      <c r="K10" t="s">
+        <v>44</v>
+      </c>
+      <c r="L10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
+      <c r="G11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
+      <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13" t="s">
+        <v>35</v>
+      </c>
+      <c r="H13" t="s">
+        <v>22</v>
+      </c>
+      <c r="I13" t="s">
+        <v>23</v>
+      </c>
+      <c r="J13" t="s">
+        <v>33</v>
+      </c>
+      <c r="K13" t="s">
+        <v>25</v>
+      </c>
+      <c r="L13" t="s">
+        <v>24</v>
+      </c>
+      <c r="M13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
+      <c r="A14">
+        <v>1</v>
+      </c>
+      <c r="B14">
+        <v>0.97512784248657902</v>
+      </c>
+      <c r="C14">
+        <f>B14*2^16</f>
+        <v>63905.978285200443</v>
+      </c>
+      <c r="D14">
+        <v>63906</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" t="s">
+        <v>36</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <v>5.7200221035302E-2</v>
+      </c>
+      <c r="J14">
+        <f>I14*2^16</f>
+        <v>3748.6736857695519</v>
+      </c>
+      <c r="K14">
+        <v>3749</v>
+      </c>
+      <c r="L14" t="s">
+        <v>49</v>
+      </c>
+      <c r="M14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
+      <c r="A15">
+        <v>2</v>
+      </c>
+      <c r="B15">
+        <v>-1.95025568497315</v>
+      </c>
+      <c r="C15">
+        <f t="shared" ref="C15:C19" si="2">B15*2^16</f>
+        <v>-127811.95657040036</v>
+      </c>
+      <c r="D15">
+        <v>-127812</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F15" t="s">
+        <v>36</v>
+      </c>
+      <c r="H15">
+        <v>2</v>
+      </c>
+      <c r="I15">
+        <v>0.114400442070604</v>
+      </c>
+      <c r="J15">
+        <f t="shared" ref="J15:J19" si="3">I15*2^16</f>
+        <v>7497.3473715391037</v>
+      </c>
+      <c r="K15">
+        <v>7497</v>
+      </c>
+      <c r="L15" t="s">
+        <v>48</v>
+      </c>
+      <c r="M15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
+      <c r="A16">
+        <v>3</v>
+      </c>
+      <c r="B16">
+        <v>0.97512784248657902</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="2"/>
+        <v>63905.978285200443</v>
+      </c>
+      <c r="D16">
+        <v>63906</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F16" t="s">
+        <v>36</v>
+      </c>
+      <c r="H16">
+        <v>3</v>
+      </c>
+      <c r="I16">
+        <v>5.7200221035302E-2</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="3"/>
+        <v>3748.6736857695519</v>
+      </c>
+      <c r="K16">
+        <v>3749</v>
+      </c>
+      <c r="L16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M16" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
+      <c r="A17">
+        <v>4</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17">
+        <f t="shared" si="2"/>
+        <v>65536</v>
+      </c>
+      <c r="D17">
+        <v>65536</v>
+      </c>
+      <c r="E17" s="3">
+        <v>10000</v>
+      </c>
+      <c r="F17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H17">
+        <v>4</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="3"/>
+        <v>65536</v>
+      </c>
+      <c r="K17">
+        <v>65536</v>
+      </c>
+      <c r="L17">
+        <v>10000</v>
+      </c>
+      <c r="M17" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
+      <c r="A18">
+        <v>5</v>
+      </c>
+      <c r="B18">
+        <v>-1.94963697662567</v>
+      </c>
+      <c r="C18">
+        <f t="shared" si="2"/>
+        <v>-127771.40890013991</v>
+      </c>
+      <c r="D18">
+        <v>-127771</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F18" t="s">
+        <v>37</v>
+      </c>
+      <c r="H18">
+        <v>5</v>
+      </c>
+      <c r="I18">
+        <v>-1.2188761083637001</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="3"/>
+        <v>-79880.264637723449</v>
+      </c>
+      <c r="K18">
+        <v>-79880</v>
+      </c>
+      <c r="L18" t="s">
+        <v>41</v>
+      </c>
+      <c r="M18" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
+      <c r="A19">
+        <v>6</v>
+      </c>
+      <c r="B19">
+        <v>0.95087439332064105</v>
+      </c>
+      <c r="C19">
+        <f t="shared" si="2"/>
+        <v>62316.504240661532</v>
+      </c>
+      <c r="D19">
+        <v>62316</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F19" t="s">
+        <v>37</v>
+      </c>
+      <c r="H19">
+        <v>6</v>
+      </c>
+      <c r="I19">
+        <v>0.447676992504908</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="3"/>
+        <v>29338.959380801651</v>
+      </c>
+      <c r="K19">
+        <v>29339</v>
+      </c>
+      <c r="L19" t="s">
+        <v>40</v>
+      </c>
+      <c r="M19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13">
+      <c r="D22" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22">
+        <v>250</v>
+      </c>
+      <c r="K22" t="s">
+        <v>43</v>
+      </c>
+      <c r="L22" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>